<commit_message>
fixed the poor performance during Request for Registers Reports on Data Base
</commit_message>
<xml_diff>
--- a/templates_formats/Info_trabajador.xlsx
+++ b/templates_formats/Info_trabajador.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Fecha:</t>
   </si>
@@ -43,9 +43,6 @@
   </si>
   <si>
     <t>CORREO:</t>
-  </si>
-  <si>
-    <t>USUARIO ASIGNADO:</t>
   </si>
   <si>
     <t>CODIGO CARGO:</t>
@@ -514,24 +511,24 @@
   <sheetData>
     <row r="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="D1" s="16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
       <c r="D2" s="17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.25">
       <c r="D3" s="18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.25">
       <c r="D4" s="19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>0</v>
@@ -539,7 +536,7 @@
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.25">
       <c r="D5" s="12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E5" s="2"/>
       <c r="H5" s="1"/>
@@ -553,7 +550,7 @@
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.25">
       <c r="D7" s="14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E7" s="2"/>
       <c r="H7" s="1"/>
@@ -610,11 +607,11 @@
       <c r="K11" s="1"/>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="D12" t="s">
+      <c r="D12" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="10" t="s">
         <v>9</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>10</v>
       </c>
       <c r="F12" s="2"/>
       <c r="H12" s="1"/>
@@ -626,10 +623,10 @@
     <row r="13" spans="2:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C13" s="7"/>
       <c r="D13" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="E13" s="11" t="s">
         <v>11</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>12</v>
       </c>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
@@ -645,10 +642,10 @@
     <row r="14" spans="2:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C14" s="7"/>
       <c r="D14" s="11" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F14" s="7"/>
       <c r="G14" s="7"/>
@@ -663,11 +660,8 @@
     </row>
     <row r="15" spans="2:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C15" s="7"/>
-      <c r="D15" s="11" t="s">
-        <v>5</v>
-      </c>
       <c r="E15" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F15" s="7"/>
       <c r="G15" s="7"/>
@@ -699,7 +693,7 @@
     <row r="17" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C17" s="7"/>
       <c r="D17" s="15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
@@ -731,10 +725,10 @@
     <row r="19" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="7"/>
       <c r="D19" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" s="11" t="s">
         <v>15</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>16</v>
       </c>
       <c r="F19" s="7"/>
       <c r="G19" s="7"/>
@@ -750,7 +744,7 @@
     <row r="20" spans="3:17" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C20" s="7"/>
       <c r="D20" s="11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E20" s="11"/>
       <c r="F20" s="7"/>

</xml_diff>